<commit_message>
feat: refine tenant threshold confirmation
</commit_message>
<xml_diff>
--- a/testcase/租户管理功能测试用例.xlsx
+++ b/testcase/租户管理功能测试用例.xlsx
@@ -590,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O70"/>
+  <dimension ref="A1:O79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4290,7 +4290,7 @@
       </c>
       <c r="K61" s="5" t="inlineStr">
         <is>
-          <t>列表与详情显示30.00、10.00，不增加任何来源或状态后缀。</t>
+          <t>列表与详情显示30.00、10.00；列表中的提醒阈值、锁定阈值和欠费锁定值后分别显示“自定义”标签。</t>
         </is>
       </c>
       <c r="L61" s="4" t="inlineStr">
@@ -4869,6 +4869,573 @@
       <c r="M70" s="7" t="n"/>
       <c r="N70" s="7" t="n"/>
       <c r="O70" s="7" t="n"/>
+    </row>
+    <row r="71" ht="58" customHeight="1">
+      <c r="A71" s="6" t="n">
+        <v>67</v>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>TEN-067</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>阈值治理</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>来源标识</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>默认租户弱化展示</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G71" s="6" t="inlineStr">
+        <is>
+          <t>界面</t>
+        </is>
+      </c>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>打开预付费项目，进入“电费相关 &gt; 分摊规则设置 &gt; 租户管理”。</t>
+        </is>
+      </c>
+      <c r="I71" s="7" t="inlineStr">
+        <is>
+          <t>存在使用项目默认阈值的租户</t>
+        </is>
+      </c>
+      <c r="J71" s="7" t="inlineStr">
+        <is>
+          <t>观察租户名称及阈值列</t>
+        </is>
+      </c>
+      <c r="K71" s="7" t="inlineStr">
+        <is>
+          <t>项目默认租户不显示额外来源标签，阈值列保持纯数值。</t>
+        </is>
+      </c>
+      <c r="L71" s="6" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="M71" s="7" t="n"/>
+      <c r="N71" s="7" t="n"/>
+      <c r="O71" s="7" t="n"/>
+    </row>
+    <row r="72" ht="58" customHeight="1">
+      <c r="A72" s="6" t="n">
+        <v>68</v>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>TEN-068</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>阈值治理</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>来源标识</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>自定义租户突出展示</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>界面</t>
+        </is>
+      </c>
+      <c r="H72" s="7" t="inlineStr">
+        <is>
+          <t>打开预付费项目，进入“电费相关 &gt; 分摊规则设置 &gt; 租户管理”。</t>
+        </is>
+      </c>
+      <c r="I72" s="7" t="inlineStr">
+        <is>
+          <t>存在单独设置阈值的租户</t>
+        </is>
+      </c>
+      <c r="J72" s="7" t="inlineStr">
+        <is>
+          <t>观察提醒阈值、锁定阈值、欠费锁定三个字段，并悬停“自定义”标签</t>
+        </is>
+      </c>
+      <c r="K72" s="7" t="inlineStr">
+        <is>
+          <t>提醒阈值、锁定阈值和欠费锁定对应值后分别显示橙色“自定义”标签；租户名称后不显示标签；悬停提示该租户不随项目默认阈值变化。</t>
+        </is>
+      </c>
+      <c r="L72" s="6" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="M72" s="7" t="n"/>
+      <c r="N72" s="7" t="n"/>
+      <c r="O72" s="7" t="n"/>
+    </row>
+    <row r="73" ht="58" customHeight="1">
+      <c r="A73" s="6" t="n">
+        <v>69</v>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>TEN-069</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>阈值治理</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>常驻提示</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>保持原有默认阈值说明</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G73" s="6" t="inlineStr">
+        <is>
+          <t>功能</t>
+        </is>
+      </c>
+      <c r="H73" s="7" t="inlineStr">
+        <is>
+          <t>打开预付费项目，进入“电费相关 &gt; 分摊规则设置 &gt; 租户管理”。</t>
+        </is>
+      </c>
+      <c r="I73" s="7" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="J73" s="7" t="inlineStr">
+        <is>
+          <t>点击“默认阈值设置”并观察弹窗常驻提示</t>
+        </is>
+      </c>
+      <c r="K73" s="7" t="inlineStr">
+        <is>
+          <t>常驻提示保持为“项目全局默认阈值：未单独配置阈值的租户默认使用此设置”，不显示影响租户数。</t>
+        </is>
+      </c>
+      <c r="L73" s="6" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="M73" s="7" t="n"/>
+      <c r="N73" s="7" t="n"/>
+      <c r="O73" s="7" t="n"/>
+    </row>
+    <row r="74" ht="58" customHeight="1">
+      <c r="A74" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>TEN-070</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>阈值治理</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>默认阈值</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>未修改不触发确认</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>功能</t>
+        </is>
+      </c>
+      <c r="H74" s="7" t="inlineStr">
+        <is>
+          <t>打开默认阈值设置弹窗。</t>
+        </is>
+      </c>
+      <c r="I74" s="7" t="inlineStr">
+        <is>
+          <t>保持提醒阈值、锁定阈值和欠费锁定状态不变</t>
+        </is>
+      </c>
+      <c r="J74" s="7" t="inlineStr">
+        <is>
+          <t>点击“提交”</t>
+        </is>
+      </c>
+      <c r="K74" s="7" t="inlineStr">
+        <is>
+          <t>提示“阈值未发生变化”，不保存且不弹出二次确认框。</t>
+        </is>
+      </c>
+      <c r="L74" s="6" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="M74" s="7" t="n"/>
+      <c r="N74" s="7" t="n"/>
+      <c r="O74" s="7" t="n"/>
+    </row>
+    <row r="75" ht="58" customHeight="1">
+      <c r="A75" s="6" t="n">
+        <v>71</v>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>TEN-071</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>阈值治理</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>二次确认</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>修改默认阈值要求确认</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G75" s="6" t="inlineStr">
+        <is>
+          <t>功能</t>
+        </is>
+      </c>
+      <c r="H75" s="7" t="inlineStr">
+        <is>
+          <t>打开默认阈值设置弹窗。</t>
+        </is>
+      </c>
+      <c r="I75" s="7" t="inlineStr">
+        <is>
+          <t>修改任一阈值或欠费锁定状态</t>
+        </is>
+      </c>
+      <c r="J75" s="7" t="inlineStr">
+        <is>
+          <t>点击“提交”</t>
+        </is>
+      </c>
+      <c r="K75" s="7" t="inlineStr">
+        <is>
+          <t>弹出二次确认，提示“本次修改将同步应用于当前项目中N 个未单独配置阈值的租户，并会按修改后的阈值对相关租户执行锁定或提醒动作。确认修改？”；N按当前项目全部租户统计，不受筛选和分页影响。</t>
+        </is>
+      </c>
+      <c r="L75" s="6" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="M75" s="7" t="n"/>
+      <c r="N75" s="7" t="n"/>
+      <c r="O75" s="7" t="n"/>
+    </row>
+    <row r="76" ht="58" customHeight="1">
+      <c r="A76" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>TEN-072</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>阈值治理</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>二次确认</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>取消后不生效</t>
+        </is>
+      </c>
+      <c r="F76" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t>功能</t>
+        </is>
+      </c>
+      <c r="H76" s="7" t="inlineStr">
+        <is>
+          <t>默认阈值已修改并打开二次确认框。</t>
+        </is>
+      </c>
+      <c r="I76" s="7" t="inlineStr">
+        <is>
+          <t>记录修改前的项目默认阈值</t>
+        </is>
+      </c>
+      <c r="J76" s="7" t="inlineStr">
+        <is>
+          <t>点击“取消”</t>
+        </is>
+      </c>
+      <c r="K76" s="7" t="inlineStr">
+        <is>
+          <t>项目默认阈值及租户生效值均不改变；编辑弹窗继续保留已输入内容。</t>
+        </is>
+      </c>
+      <c r="L76" s="6" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="M76" s="7" t="n"/>
+      <c r="N76" s="7" t="n"/>
+      <c r="O76" s="7" t="n"/>
+    </row>
+    <row r="77" ht="58" customHeight="1">
+      <c r="A77" s="6" t="n">
+        <v>73</v>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>TEN-073</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>阈值治理</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>同步生效</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>确认后仅更新跟随租户</t>
+        </is>
+      </c>
+      <c r="F77" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G77" s="6" t="inlineStr">
+        <is>
+          <t>功能</t>
+        </is>
+      </c>
+      <c r="H77" s="7" t="inlineStr">
+        <is>
+          <t>默认阈值已修改并打开二次确认框。</t>
+        </is>
+      </c>
+      <c r="I77" s="7" t="inlineStr">
+        <is>
+          <t>同时存在项目默认租户和自定义租户</t>
+        </is>
+      </c>
+      <c r="J77" s="7" t="inlineStr">
+        <is>
+          <t>点击“确定”并观察两类租户</t>
+        </is>
+      </c>
+      <c r="K77" s="7" t="inlineStr">
+        <is>
+          <t>项目默认租户同步使用新阈值；自定义租户保持原值不变。</t>
+        </is>
+      </c>
+      <c r="L77" s="6" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="M77" s="7" t="n"/>
+      <c r="N77" s="7" t="n"/>
+      <c r="O77" s="7" t="n"/>
+    </row>
+    <row r="78" ht="58" customHeight="1">
+      <c r="A78" s="6" t="n">
+        <v>74</v>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>TEN-074</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>阈值治理</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>恢复默认</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>恢复入口仅对自定义租户显示</t>
+        </is>
+      </c>
+      <c r="F78" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G78" s="6" t="inlineStr">
+        <is>
+          <t>界面</t>
+        </is>
+      </c>
+      <c r="H78" s="7" t="inlineStr">
+        <is>
+          <t>打开预付费项目租户管理。</t>
+        </is>
+      </c>
+      <c r="I78" s="7" t="inlineStr">
+        <is>
+          <t>分别选择项目默认租户和自定义租户</t>
+        </is>
+      </c>
+      <c r="J78" s="7" t="inlineStr">
+        <is>
+          <t>依次打开单租户“阈值设置”弹窗</t>
+        </is>
+      </c>
+      <c r="K78" s="7" t="inlineStr">
+        <is>
+          <t>自定义租户显示“恢复项目默认值”；项目默认租户不显示该入口。</t>
+        </is>
+      </c>
+      <c r="L78" s="6" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="M78" s="7" t="n"/>
+      <c r="N78" s="7" t="n"/>
+      <c r="O78" s="7" t="n"/>
+    </row>
+    <row r="79" ht="58" customHeight="1">
+      <c r="A79" s="6" t="n">
+        <v>75</v>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>TEN-075</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>阈值治理</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>恢复默认</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>确认恢复后重新跟随项目默认值</t>
+        </is>
+      </c>
+      <c r="F79" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G79" s="6" t="inlineStr">
+        <is>
+          <t>功能</t>
+        </is>
+      </c>
+      <c r="H79" s="7" t="inlineStr">
+        <is>
+          <t>打开自定义租户的阈值设置弹窗。</t>
+        </is>
+      </c>
+      <c r="I79" s="7" t="inlineStr">
+        <is>
+          <t>当前项目默认阈值与该租户自定义阈值不同</t>
+        </is>
+      </c>
+      <c r="J79" s="7" t="inlineStr">
+        <is>
+          <t>点击“恢复项目默认值”并确认</t>
+        </is>
+      </c>
+      <c r="K79" s="7" t="inlineStr">
+        <is>
+          <t>清除该租户自定义状态和“自定义”标签，立即使用当前项目默认阈值，之后继续跟随项目默认值变化。</t>
+        </is>
+      </c>
+      <c r="L79" s="6" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="M79" s="7" t="n"/>
+      <c r="N79" s="7" t="n"/>
+      <c r="O79" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:O70"/>
@@ -4929,7 +5496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5016,7 +5583,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>75</t>
         </is>
       </c>
       <c r="C6" s="11" t="n"/>
@@ -5096,7 +5663,7 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>租户名称、联系人名称；阈值纯数值；租户ID；欠费锁定列；余额无文字备注</t>
+          <t>租户名称、联系人名称；阈值数值；租户ID；欠费锁定列；余额无文字备注；三个阈值相关字段的自定义标签</t>
         </is>
       </c>
       <c r="C12" s="11" t="n"/>
@@ -5183,6 +5750,22 @@
       <c r="D17" s="11" t="n"/>
       <c r="E17" s="11" t="n"/>
       <c r="F17" s="12" t="n"/>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>阈值治理</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>项目默认持续跟随、自定义例外标识、常驻说明、保存时影响面提示、二次确认、未变化拦截、恢复项目默认值</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">

</xml_diff>